<commit_message>
Added 36v TVS diode
</commit_message>
<xml_diff>
--- a/To Add v2/Protection - TVS Diode.xlsx
+++ b/To Add v2/Protection - TVS Diode.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\To Add v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11207046-2C2E-49FC-A063-21922466A010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F035DAB2-14EC-414C-B189-3FF8E7144173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="7725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="57">
   <si>
     <t>Totals</t>
   </si>
@@ -152,9 +152,6 @@
     <t>Uni</t>
   </si>
   <si>
-    <t>BAV99</t>
-  </si>
-  <si>
     <t>Steering</t>
   </si>
   <si>
@@ -189,6 +186,27 @@
   </si>
   <si>
     <t>Diodes:D_0201_0603Metric</t>
+  </si>
+  <si>
+    <t>SMBJ36CA-13-F</t>
+  </si>
+  <si>
+    <t>Bidir</t>
+  </si>
+  <si>
+    <t>SMB</t>
+  </si>
+  <si>
+    <t>SMBJ36CA-FDICT-ND</t>
+  </si>
+  <si>
+    <t>https://www.diodes.com/assets/Datasheets/ds19002.pdf</t>
+  </si>
+  <si>
+    <t>0Dan_Protection_D_TVS_Dual</t>
+  </si>
+  <si>
+    <t>Diodes:D_SMB_Bidir</t>
   </si>
 </sst>
 </file>
@@ -250,7 +268,15 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -526,103 +552,103 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:AB9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="43.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="2"/>
-    <col min="13" max="13" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
-    <col min="15" max="15" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.90625" style="2"/>
+    <col min="13" max="13" width="17.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.36328125" customWidth="1"/>
+    <col min="15" max="15" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.81640625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="25" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="19" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B1" s="1"/>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="2:28" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2">
         <f>COUNTA(C7:C9999)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:T2" si="0">COUNTA(D7:D9999)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2">
         <f t="shared" ref="F2" si="1">COUNTA(F7:F9999)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2">
         <f t="shared" ref="G2:L2" si="2">COUNTA(G7:G9999)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J2">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L2">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T2">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AA2" t="s">
         <v>1</v>
@@ -632,17 +658,17 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="2:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:28" x14ac:dyDescent="0.35">
       <c r="L3"/>
       <c r="AA3" t="s">
         <v>2</v>
       </c>
       <c r="AB3">
         <f>MAX(C2:T2)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -708,7 +734,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:28" x14ac:dyDescent="0.35">
       <c r="AA5" t="s">
         <v>5</v>
       </c>
@@ -717,7 +743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:28" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>6</v>
       </c>
@@ -782,7 +808,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:28" x14ac:dyDescent="0.35">
       <c r="C7" t="str">
         <f>_xlfn.CONCAT(D7," ",I7,"A ",L7," ",T7)</f>
         <v>Zener 1Ch Uni 5.5V 11A 0201 Orentation Unverified</v>
@@ -831,13 +857,13 @@
         <v>27</v>
       </c>
       <c r="R7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="T7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="W7">
         <f>COUNTBLANK(C7:T7)</f>
@@ -859,16 +885,17 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="2:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:28" x14ac:dyDescent="0.35">
       <c r="C8" t="str">
         <f>_xlfn.CONCAT(D8," ",I8,"A ",L8," ",T8)</f>
-        <v>BAV99 2A SOT23-3  </v>
-      </c>
-      <c r="D8" t="s">
+        <v>Steering 1Ch    V 2A SOT23-3  </v>
+      </c>
+      <c r="D8" t="str">
+        <f t="shared" ref="D8:D9" si="3">_xlfn.CONCAT(E8," ",F8,"Ch ",G8," ",H8,"V")</f>
+        <v>Steering 1Ch    V</v>
+      </c>
+      <c r="E8" t="s">
         <v>38</v>
-      </c>
-      <c r="E8" t="s">
-        <v>39</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -886,31 +913,31 @@
         <v>35</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="N8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O8" t="s">
         <v>25</v>
       </c>
       <c r="P8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="R8" t="s">
+        <v>46</v>
+      </c>
+      <c r="S8" t="s">
         <v>47</v>
-      </c>
-      <c r="S8" t="s">
-        <v>48</v>
       </c>
       <c r="T8" t="s">
         <v>35</v>
@@ -928,7 +955,70 @@
         <v>1</v>
       </c>
     </row>
+    <row r="9" spans="2:28" x14ac:dyDescent="0.35">
+      <c r="C9" t="str">
+        <f>_xlfn.CONCAT(D9," ",I9,"A ",L9," ",T9)</f>
+        <v>Zener 1Ch Bidir 36V 10.3A SMB  </v>
+      </c>
+      <c r="D9" t="str">
+        <f t="shared" si="3"/>
+        <v>Zener 1Ch Bidir 36V</v>
+      </c>
+      <c r="E9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9">
+        <v>36</v>
+      </c>
+      <c r="I9">
+        <v>10.3</v>
+      </c>
+      <c r="J9">
+        <v>600</v>
+      </c>
+      <c r="K9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="M9" t="s">
+        <v>41</v>
+      </c>
+      <c r="N9" t="s">
+        <v>50</v>
+      </c>
+      <c r="O9" t="s">
+        <v>25</v>
+      </c>
+      <c r="P9" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>54</v>
+      </c>
+      <c r="R9" t="s">
+        <v>55</v>
+      </c>
+      <c r="S9" t="s">
+        <v>56</v>
+      </c>
+      <c r="T9" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C7:T41">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(C7))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="K7" r:id="rId1" xr:uid="{5D8C1057-12A4-42D0-A591-2242E50146B9}"/>
     <hyperlink ref="K8" r:id="rId2" xr:uid="{41297C62-6D6E-42EF-9ABA-3CFEE4736466}"/>

</xml_diff>